<commit_message>
Complete N100 financial intelligence deliverables
</commit_message>
<xml_diff>
--- a/N100 FINANCIAL INTELLIGENCE PLATFORM/output/valuation_summary.xlsx
+++ b/N100 FINANCIAL INTELLIGENCE PLATFORM/output/valuation_summary.xlsx
@@ -1,14 +1,420 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="valuation_summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J93"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -78,22 +484,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>17.47</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>1.48</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>12.46</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>6.05</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="n">
         <v>16.91</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="n">
         <v>-27.87</v>
       </c>
       <c r="J2" t="inlineStr">
@@ -118,22 +524,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>18.82</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>1.76</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>13.6</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>6.94</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="n">
         <v>18.26</v>
       </c>
-      <c r="I3">
+      <c r="I3" t="n">
         <v>-22.3</v>
       </c>
       <c r="J3" t="inlineStr">
@@ -158,22 +564,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>20.17</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>2.04</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>14.75</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>8.1</v>
       </c>
-      <c r="H4">
+      <c r="H4" t="n">
         <v>19.61</v>
       </c>
-      <c r="I4">
+      <c r="I4" t="n">
         <v>-21.12</v>
       </c>
       <c r="J4" t="inlineStr">
@@ -198,22 +604,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>21.52</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>2.32</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>15.89</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>9.15</v>
       </c>
-      <c r="H5">
+      <c r="H5" t="n">
         <v>20.96</v>
       </c>
-      <c r="I5">
+      <c r="I5" t="n">
         <v>-20.06</v>
       </c>
       <c r="J5" t="inlineStr">
@@ -238,22 +644,22 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>22.87</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>2.6</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>17.04</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>6.26</v>
       </c>
-      <c r="H6">
+      <c r="H6" t="n">
         <v>22.31</v>
       </c>
-      <c r="I6">
+      <c r="I6" t="n">
         <v>-20.99</v>
       </c>
       <c r="J6" t="inlineStr">
@@ -278,22 +684,22 @@
           <t>Automobile</t>
         </is>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>24.22</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>2.88</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>18.18</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>6.48</v>
       </c>
-      <c r="H7">
+      <c r="H7" t="n">
         <v>23.66</v>
       </c>
-      <c r="I7">
+      <c r="I7" t="n">
         <v>-10.03</v>
       </c>
       <c r="J7" t="inlineStr">
@@ -318,22 +724,22 @@
           <t>Metals</t>
         </is>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>25.57</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>3.16</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>19.33</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>4.9</v>
       </c>
-      <c r="H8">
+      <c r="H8" t="n">
         <v>25.01</v>
       </c>
-      <c r="I8">
+      <c r="I8" t="n">
         <v>2.71</v>
       </c>
       <c r="J8" t="inlineStr">
@@ -358,23 +764,23 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>26.92</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>3.44</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>20.47</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>4.83</v>
       </c>
-      <c r="H9">
+      <c r="H9" t="n">
         <v>26.36</v>
       </c>
-      <c r="I9">
-        <v>8.13</v>
+      <c r="I9" t="n">
+        <v>8.130000000000001</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -398,22 +804,22 @@
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>28.27</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>3.72</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>21.62</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>4.99</v>
       </c>
-      <c r="H10">
+      <c r="H10" t="n">
         <v>27.71</v>
       </c>
-      <c r="I10">
+      <c r="I10" t="n">
         <v>7.72</v>
       </c>
       <c r="J10" t="inlineStr">
@@ -438,22 +844,22 @@
           <t>Telecom</t>
         </is>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>29.62</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>4</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>22.76</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>3.56</v>
       </c>
-      <c r="H11">
+      <c r="H11" t="n">
         <v>29.06</v>
       </c>
-      <c r="I11">
+      <c r="I11" t="n">
         <v>7.34</v>
       </c>
       <c r="J11" t="inlineStr">
@@ -478,22 +884,22 @@
           <t>Chemicals</t>
         </is>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>30.97</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>4.28</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>23.91</v>
       </c>
-      <c r="G12">
-        <v>4.3</v>
-      </c>
-      <c r="H12">
+      <c r="G12" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="H12" t="n">
         <v>30.41</v>
       </c>
-      <c r="I12">
+      <c r="I12" t="n">
         <v>7</v>
       </c>
       <c r="J12" t="inlineStr">
@@ -518,22 +924,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>32.32</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>4.56</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>25.05</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>5.15</v>
       </c>
-      <c r="H13">
+      <c r="H13" t="n">
         <v>31.76</v>
       </c>
-      <c r="I13">
+      <c r="I13" t="n">
         <v>33.44</v>
       </c>
       <c r="J13" t="inlineStr">
@@ -558,22 +964,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>33.67</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>1.2</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>22.2</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>5.87</v>
       </c>
-      <c r="H14">
+      <c r="H14" t="n">
         <v>33.11</v>
       </c>
-      <c r="I14">
+      <c r="I14" t="n">
         <v>39.02</v>
       </c>
       <c r="J14" t="inlineStr">
@@ -598,22 +1004,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>35.02</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>1.48</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>23.34</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>4.8</v>
       </c>
-      <c r="H15">
+      <c r="H15" t="n">
         <v>34.46</v>
       </c>
-      <c r="I15">
+      <c r="I15" t="n">
         <v>36.96</v>
       </c>
       <c r="J15" t="inlineStr">
@@ -638,22 +1044,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>36.37</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>1.76</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="n">
         <v>24.49</v>
       </c>
-      <c r="G16">
+      <c r="G16" t="n">
         <v>3.12</v>
       </c>
-      <c r="H16">
+      <c r="H16" t="n">
         <v>35.81</v>
       </c>
-      <c r="I16">
+      <c r="I16" t="n">
         <v>35.1</v>
       </c>
       <c r="J16" t="inlineStr">
@@ -678,22 +1084,22 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D17">
+      <c r="D17" t="n">
         <v>37.72</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="n">
         <v>2.04</v>
       </c>
-      <c r="F17">
+      <c r="F17" t="n">
         <v>25.63</v>
       </c>
-      <c r="G17">
+      <c r="G17" t="n">
         <v>3.15</v>
       </c>
-      <c r="H17">
+      <c r="H17" t="n">
         <v>37.16</v>
       </c>
-      <c r="I17">
+      <c r="I17" t="n">
         <v>30.32</v>
       </c>
       <c r="J17" t="inlineStr">
@@ -718,22 +1124,22 @@
           <t>Automobile</t>
         </is>
       </c>
-      <c r="D18">
+      <c r="D18" t="n">
         <v>16.12</v>
       </c>
-      <c r="E18">
+      <c r="E18" t="n">
         <v>2.32</v>
       </c>
-      <c r="F18">
+      <c r="F18" t="n">
         <v>12.55</v>
       </c>
-      <c r="G18">
+      <c r="G18" t="n">
         <v>7.82</v>
       </c>
-      <c r="H18">
+      <c r="H18" t="n">
         <v>15.56</v>
       </c>
-      <c r="I18">
+      <c r="I18" t="n">
         <v>-40.12</v>
       </c>
       <c r="J18" t="inlineStr">
@@ -758,22 +1164,22 @@
           <t>Metals</t>
         </is>
       </c>
-      <c r="D19">
+      <c r="D19" t="n">
         <v>17.47</v>
       </c>
-      <c r="E19">
+      <c r="E19" t="n">
         <v>2.6</v>
       </c>
-      <c r="F19">
+      <c r="F19" t="n">
         <v>13.69</v>
       </c>
-      <c r="G19">
+      <c r="G19" t="n">
         <v>8.09</v>
       </c>
-      <c r="H19">
+      <c r="H19" t="n">
         <v>16.91</v>
       </c>
-      <c r="I19">
+      <c r="I19" t="n">
         <v>-29.83</v>
       </c>
       <c r="J19" t="inlineStr">
@@ -798,22 +1204,22 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D20">
+      <c r="D20" t="n">
         <v>18.82</v>
       </c>
-      <c r="E20">
+      <c r="E20" t="n">
         <v>2.88</v>
       </c>
-      <c r="F20">
+      <c r="F20" t="n">
         <v>14.84</v>
       </c>
-      <c r="G20">
+      <c r="G20" t="n">
         <v>9</v>
       </c>
-      <c r="H20">
+      <c r="H20" t="n">
         <v>18.26</v>
       </c>
-      <c r="I20">
+      <c r="I20" t="n">
         <v>-24.4</v>
       </c>
       <c r="J20" t="inlineStr">
@@ -838,22 +1244,22 @@
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="D21">
+      <c r="D21" t="n">
         <v>20.17</v>
       </c>
-      <c r="E21">
+      <c r="E21" t="n">
         <v>3.16</v>
       </c>
-      <c r="F21">
+      <c r="F21" t="n">
         <v>15.98</v>
       </c>
-      <c r="G21">
+      <c r="G21" t="n">
         <v>6.64</v>
       </c>
-      <c r="H21">
+      <c r="H21" t="n">
         <v>19.61</v>
       </c>
-      <c r="I21">
+      <c r="I21" t="n">
         <v>-23.15</v>
       </c>
       <c r="J21" t="inlineStr">
@@ -878,22 +1284,22 @@
           <t>Telecom</t>
         </is>
       </c>
-      <c r="D22">
+      <c r="D22" t="n">
         <v>21.52</v>
       </c>
-      <c r="E22">
+      <c r="E22" t="n">
         <v>3.44</v>
       </c>
-      <c r="F22">
+      <c r="F22" t="n">
         <v>17.13</v>
       </c>
-      <c r="G22">
+      <c r="G22" t="n">
         <v>5.94</v>
       </c>
-      <c r="H22">
+      <c r="H22" t="n">
         <v>20.96</v>
       </c>
-      <c r="I22">
+      <c r="I22" t="n">
         <v>-22.01</v>
       </c>
       <c r="J22" t="inlineStr">
@@ -918,22 +1324,22 @@
           <t>Chemicals</t>
         </is>
       </c>
-      <c r="D23">
+      <c r="D23" t="n">
         <v>22.87</v>
       </c>
-      <c r="E23">
+      <c r="E23" t="n">
         <v>3.72</v>
       </c>
-      <c r="F23">
+      <c r="F23" t="n">
         <v>18.27</v>
       </c>
-      <c r="G23">
+      <c r="G23" t="n">
         <v>6.58</v>
       </c>
-      <c r="H23">
+      <c r="H23" t="n">
         <v>22.31</v>
       </c>
-      <c r="I23">
+      <c r="I23" t="n">
         <v>-20.99</v>
       </c>
       <c r="J23" t="inlineStr">
@@ -958,22 +1364,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D24">
+      <c r="D24" t="n">
         <v>24.22</v>
       </c>
-      <c r="E24">
+      <c r="E24" t="n">
         <v>4</v>
       </c>
-      <c r="F24">
+      <c r="F24" t="n">
         <v>19.42</v>
       </c>
-      <c r="G24">
+      <c r="G24" t="n">
         <v>6.81</v>
       </c>
-      <c r="H24">
+      <c r="H24" t="n">
         <v>23.66</v>
       </c>
-      <c r="I24">
+      <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="inlineStr">
@@ -998,22 +1404,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D25">
+      <c r="D25" t="n">
         <v>25.57</v>
       </c>
-      <c r="E25">
+      <c r="E25" t="n">
         <v>4.28</v>
       </c>
-      <c r="F25">
+      <c r="F25" t="n">
         <v>20.56</v>
       </c>
-      <c r="G25">
+      <c r="G25" t="n">
         <v>6.68</v>
       </c>
-      <c r="H25">
+      <c r="H25" t="n">
         <v>25.01</v>
       </c>
-      <c r="I25">
+      <c r="I25" t="n">
         <v>5.57</v>
       </c>
       <c r="J25" t="inlineStr">
@@ -1038,22 +1444,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D26">
+      <c r="D26" t="n">
         <v>26.92</v>
       </c>
-      <c r="E26">
+      <c r="E26" t="n">
         <v>4.56</v>
       </c>
-      <c r="F26">
+      <c r="F26" t="n">
         <v>21.71</v>
       </c>
-      <c r="G26">
+      <c r="G26" t="n">
         <v>4.14</v>
       </c>
-      <c r="H26">
+      <c r="H26" t="n">
         <v>26.36</v>
       </c>
-      <c r="I26">
+      <c r="I26" t="n">
         <v>5.28</v>
       </c>
       <c r="J26" t="inlineStr">
@@ -1078,22 +1484,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D27">
+      <c r="D27" t="n">
         <v>28.27</v>
       </c>
-      <c r="E27">
+      <c r="E27" t="n">
         <v>1.2</v>
       </c>
-      <c r="F27">
+      <c r="F27" t="n">
         <v>18.85</v>
       </c>
-      <c r="G27">
+      <c r="G27" t="n">
         <v>4.3</v>
       </c>
-      <c r="H27">
+      <c r="H27" t="n">
         <v>27.71</v>
       </c>
-      <c r="I27">
+      <c r="I27" t="n">
         <v>5.01</v>
       </c>
       <c r="J27" t="inlineStr">
@@ -1118,22 +1524,22 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D28">
+      <c r="D28" t="n">
         <v>29.62</v>
       </c>
-      <c r="E28">
+      <c r="E28" t="n">
         <v>1.48</v>
       </c>
-      <c r="F28">
+      <c r="F28" t="n">
         <v>19.99</v>
       </c>
-      <c r="G28">
+      <c r="G28" t="n">
         <v>4.78</v>
       </c>
-      <c r="H28">
+      <c r="H28" t="n">
         <v>29.06</v>
       </c>
-      <c r="I28">
+      <c r="I28" t="n">
         <v>2.33</v>
       </c>
       <c r="J28" t="inlineStr">
@@ -1158,22 +1564,22 @@
           <t>Automobile</t>
         </is>
       </c>
-      <c r="D29">
+      <c r="D29" t="n">
         <v>30.97</v>
       </c>
-      <c r="E29">
+      <c r="E29" t="n">
         <v>1.76</v>
       </c>
-      <c r="F29">
+      <c r="F29" t="n">
         <v>21.14</v>
       </c>
-      <c r="G29">
+      <c r="G29" t="n">
         <v>4.31</v>
       </c>
-      <c r="H29">
+      <c r="H29" t="n">
         <v>30.41</v>
       </c>
-      <c r="I29">
+      <c r="I29" t="n">
         <v>15.04</v>
       </c>
       <c r="J29" t="inlineStr">
@@ -1198,22 +1604,22 @@
           <t>Metals</t>
         </is>
       </c>
-      <c r="D30">
+      <c r="D30" t="n">
         <v>32.32</v>
       </c>
-      <c r="E30">
+      <c r="E30" t="n">
         <v>2.04</v>
       </c>
-      <c r="F30">
+      <c r="F30" t="n">
         <v>22.28</v>
       </c>
-      <c r="G30">
+      <c r="G30" t="n">
         <v>5.14</v>
       </c>
-      <c r="H30">
+      <c r="H30" t="n">
         <v>31.76</v>
       </c>
-      <c r="I30">
+      <c r="I30" t="n">
         <v>29.83</v>
       </c>
       <c r="J30" t="inlineStr">
@@ -1238,22 +1644,22 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D31">
+      <c r="D31" t="n">
         <v>33.67</v>
       </c>
-      <c r="E31">
+      <c r="E31" t="n">
         <v>2.32</v>
       </c>
-      <c r="F31">
+      <c r="F31" t="n">
         <v>23.43</v>
       </c>
-      <c r="G31">
+      <c r="G31" t="n">
         <v>3.78</v>
       </c>
-      <c r="H31">
+      <c r="H31" t="n">
         <v>33.11</v>
       </c>
-      <c r="I31">
+      <c r="I31" t="n">
         <v>35.25</v>
       </c>
       <c r="J31" t="inlineStr">
@@ -1278,22 +1684,22 @@
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="D32">
+      <c r="D32" t="n">
         <v>35.02</v>
       </c>
-      <c r="E32">
+      <c r="E32" t="n">
         <v>2.6</v>
       </c>
-      <c r="F32">
+      <c r="F32" t="n">
         <v>24.57</v>
       </c>
-      <c r="G32">
+      <c r="G32" t="n">
         <v>4.2</v>
       </c>
-      <c r="H32">
+      <c r="H32" t="n">
         <v>34.46</v>
       </c>
-      <c r="I32">
+      <c r="I32" t="n">
         <v>33.43</v>
       </c>
       <c r="J32" t="inlineStr">
@@ -1318,22 +1724,22 @@
           <t>Telecom</t>
         </is>
       </c>
-      <c r="D33">
+      <c r="D33" t="n">
         <v>36.37</v>
       </c>
-      <c r="E33">
+      <c r="E33" t="n">
         <v>2.88</v>
       </c>
-      <c r="F33">
+      <c r="F33" t="n">
         <v>25.72</v>
       </c>
-      <c r="G33">
+      <c r="G33" t="n">
         <v>4.36</v>
       </c>
-      <c r="H33">
+      <c r="H33" t="n">
         <v>35.81</v>
       </c>
-      <c r="I33">
+      <c r="I33" t="n">
         <v>31.8</v>
       </c>
       <c r="J33" t="inlineStr">
@@ -1358,22 +1764,22 @@
           <t>Chemicals</t>
         </is>
       </c>
-      <c r="D34">
+      <c r="D34" t="n">
         <v>37.72</v>
       </c>
-      <c r="E34">
+      <c r="E34" t="n">
         <v>3.16</v>
       </c>
-      <c r="F34">
+      <c r="F34" t="n">
         <v>26.86</v>
       </c>
-      <c r="G34">
+      <c r="G34" t="n">
         <v>4.33</v>
       </c>
-      <c r="H34">
+      <c r="H34" t="n">
         <v>37.16</v>
       </c>
-      <c r="I34">
+      <c r="I34" t="n">
         <v>30.32</v>
       </c>
       <c r="J34" t="inlineStr">
@@ -1398,22 +1804,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D35">
+      <c r="D35" t="n">
         <v>16.12</v>
       </c>
-      <c r="E35">
+      <c r="E35" t="n">
         <v>3.44</v>
       </c>
-      <c r="F35">
+      <c r="F35" t="n">
         <v>13.78</v>
       </c>
-      <c r="G35">
+      <c r="G35" t="n">
         <v>10.42</v>
       </c>
-      <c r="H35">
+      <c r="H35" t="n">
         <v>15.56</v>
       </c>
-      <c r="I35">
+      <c r="I35" t="n">
         <v>-33.44</v>
       </c>
       <c r="J35" t="inlineStr">
@@ -1438,22 +1844,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D36">
+      <c r="D36" t="n">
         <v>17.47</v>
       </c>
-      <c r="E36">
+      <c r="E36" t="n">
         <v>3.72</v>
       </c>
-      <c r="F36">
+      <c r="F36" t="n">
         <v>14.92</v>
       </c>
-      <c r="G36">
+      <c r="G36" t="n">
         <v>5.15</v>
       </c>
-      <c r="H36">
+      <c r="H36" t="n">
         <v>16.91</v>
       </c>
-      <c r="I36">
+      <c r="I36" t="n">
         <v>-27.87</v>
       </c>
       <c r="J36" t="inlineStr">
@@ -1478,22 +1884,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D37">
+      <c r="D37" t="n">
         <v>18.82</v>
       </c>
-      <c r="E37">
+      <c r="E37" t="n">
         <v>4</v>
       </c>
-      <c r="F37">
+      <c r="F37" t="n">
         <v>16.07</v>
       </c>
-      <c r="G37">
+      <c r="G37" t="n">
         <v>5.83</v>
       </c>
-      <c r="H37">
+      <c r="H37" t="n">
         <v>18.26</v>
       </c>
-      <c r="I37">
+      <c r="I37" t="n">
         <v>-26.4</v>
       </c>
       <c r="J37" t="inlineStr">
@@ -1518,22 +1924,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D38">
+      <c r="D38" t="n">
         <v>20.17</v>
       </c>
-      <c r="E38">
+      <c r="E38" t="n">
         <v>4.28</v>
       </c>
-      <c r="F38">
+      <c r="F38" t="n">
         <v>17.21</v>
       </c>
-      <c r="G38">
+      <c r="G38" t="n">
         <v>6.86</v>
       </c>
-      <c r="H38">
+      <c r="H38" t="n">
         <v>19.61</v>
       </c>
-      <c r="I38">
+      <c r="I38" t="n">
         <v>-25.07</v>
       </c>
       <c r="J38" t="inlineStr">
@@ -1558,22 +1964,22 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D39">
+      <c r="D39" t="n">
         <v>21.52</v>
       </c>
-      <c r="E39">
+      <c r="E39" t="n">
         <v>4.56</v>
       </c>
-      <c r="F39">
+      <c r="F39" t="n">
         <v>18.36</v>
       </c>
-      <c r="G39">
+      <c r="G39" t="n">
         <v>7.94</v>
       </c>
-      <c r="H39">
+      <c r="H39" t="n">
         <v>20.96</v>
       </c>
-      <c r="I39">
+      <c r="I39" t="n">
         <v>-25.65</v>
       </c>
       <c r="J39" t="inlineStr">
@@ -1598,22 +2004,22 @@
           <t>Automobile</t>
         </is>
       </c>
-      <c r="D40">
+      <c r="D40" t="n">
         <v>22.87</v>
       </c>
-      <c r="E40">
+      <c r="E40" t="n">
         <v>1.2</v>
       </c>
-      <c r="F40">
+      <c r="F40" t="n">
         <v>15.5</v>
       </c>
-      <c r="G40">
+      <c r="G40" t="n">
         <v>8.74</v>
       </c>
-      <c r="H40">
+      <c r="H40" t="n">
         <v>22.31</v>
       </c>
-      <c r="I40">
+      <c r="I40" t="n">
         <v>-15.04</v>
       </c>
       <c r="J40" t="inlineStr">
@@ -1638,22 +2044,22 @@
           <t>Metals</t>
         </is>
       </c>
-      <c r="D41">
+      <c r="D41" t="n">
         <v>24.22</v>
       </c>
-      <c r="E41">
+      <c r="E41" t="n">
         <v>1.48</v>
       </c>
-      <c r="F41">
+      <c r="F41" t="n">
         <v>16.64</v>
       </c>
-      <c r="G41">
+      <c r="G41" t="n">
         <v>5.79</v>
       </c>
-      <c r="H41">
+      <c r="H41" t="n">
         <v>23.66</v>
       </c>
-      <c r="I41">
+      <c r="I41" t="n">
         <v>-2.71</v>
       </c>
       <c r="J41" t="inlineStr">
@@ -1678,22 +2084,22 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D42">
+      <c r="D42" t="n">
         <v>25.57</v>
       </c>
-      <c r="E42">
+      <c r="E42" t="n">
         <v>1.76</v>
       </c>
-      <c r="F42">
+      <c r="F42" t="n">
         <v>17.79</v>
       </c>
-      <c r="G42">
+      <c r="G42" t="n">
         <v>5.85</v>
       </c>
-      <c r="H42">
+      <c r="H42" t="n">
         <v>25.01</v>
       </c>
-      <c r="I42">
+      <c r="I42" t="n">
         <v>2.71</v>
       </c>
       <c r="J42" t="inlineStr">
@@ -1718,22 +2124,22 @@
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="D43">
+      <c r="D43" t="n">
         <v>26.92</v>
       </c>
-      <c r="E43">
+      <c r="E43" t="n">
         <v>2.04</v>
       </c>
-      <c r="F43">
+      <c r="F43" t="n">
         <v>18.93</v>
       </c>
-      <c r="G43">
+      <c r="G43" t="n">
         <v>4.4</v>
       </c>
-      <c r="H43">
+      <c r="H43" t="n">
         <v>26.36</v>
       </c>
-      <c r="I43">
+      <c r="I43" t="n">
         <v>2.57</v>
       </c>
       <c r="J43" t="inlineStr">
@@ -1758,22 +2164,22 @@
           <t>Telecom</t>
         </is>
       </c>
-      <c r="D44">
+      <c r="D44" t="n">
         <v>28.27</v>
       </c>
-      <c r="E44">
+      <c r="E44" t="n">
         <v>2.32</v>
       </c>
-      <c r="F44">
+      <c r="F44" t="n">
         <v>20.08</v>
       </c>
-      <c r="G44">
+      <c r="G44" t="n">
         <v>4.46</v>
       </c>
-      <c r="H44">
+      <c r="H44" t="n">
         <v>27.71</v>
       </c>
-      <c r="I44">
+      <c r="I44" t="n">
         <v>2.45</v>
       </c>
       <c r="J44" t="inlineStr">
@@ -1798,22 +2204,22 @@
           <t>Chemicals</t>
         </is>
       </c>
-      <c r="D45">
+      <c r="D45" t="n">
         <v>29.62</v>
       </c>
-      <c r="E45">
+      <c r="E45" t="n">
         <v>2.6</v>
       </c>
-      <c r="F45">
+      <c r="F45" t="n">
         <v>21.22</v>
       </c>
-      <c r="G45">
+      <c r="G45" t="n">
         <v>4.82</v>
       </c>
-      <c r="H45">
+      <c r="H45" t="n">
         <v>29.06</v>
       </c>
-      <c r="I45">
+      <c r="I45" t="n">
         <v>2.33</v>
       </c>
       <c r="J45" t="inlineStr">
@@ -1838,22 +2244,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D46">
+      <c r="D46" t="n">
         <v>30.97</v>
       </c>
-      <c r="E46">
+      <c r="E46" t="n">
         <v>2.88</v>
       </c>
-      <c r="F46">
+      <c r="F46" t="n">
         <v>22.37</v>
       </c>
-      <c r="G46">
+      <c r="G46" t="n">
         <v>3.58</v>
       </c>
-      <c r="H46">
+      <c r="H46" t="n">
         <v>30.41</v>
       </c>
-      <c r="I46">
+      <c r="I46" t="n">
         <v>27.87</v>
       </c>
       <c r="J46" t="inlineStr">
@@ -1878,22 +2284,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D47">
+      <c r="D47" t="n">
         <v>32.32</v>
       </c>
-      <c r="E47">
+      <c r="E47" t="n">
         <v>3.16</v>
       </c>
-      <c r="F47">
+      <c r="F47" t="n">
         <v>23.51</v>
       </c>
-      <c r="G47">
+      <c r="G47" t="n">
         <v>4.36</v>
       </c>
-      <c r="H47">
+      <c r="H47" t="n">
         <v>31.76</v>
       </c>
-      <c r="I47">
+      <c r="I47" t="n">
         <v>33.44</v>
       </c>
       <c r="J47" t="inlineStr">
@@ -1918,22 +2324,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D48">
+      <c r="D48" t="n">
         <v>33.67</v>
       </c>
-      <c r="E48">
+      <c r="E48" t="n">
         <v>3.44</v>
       </c>
-      <c r="F48">
+      <c r="F48" t="n">
         <v>24.66</v>
       </c>
-      <c r="G48">
+      <c r="G48" t="n">
         <v>5.12</v>
       </c>
-      <c r="H48">
+      <c r="H48" t="n">
         <v>33.11</v>
       </c>
-      <c r="I48">
+      <c r="I48" t="n">
         <v>31.68</v>
       </c>
       <c r="J48" t="inlineStr">
@@ -1958,22 +2364,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D49">
+      <c r="D49" t="n">
         <v>35.02</v>
       </c>
-      <c r="E49">
+      <c r="E49" t="n">
         <v>3.72</v>
       </c>
-      <c r="F49">
+      <c r="F49" t="n">
         <v>25.8</v>
       </c>
-      <c r="G49">
+      <c r="G49" t="n">
         <v>5.65</v>
       </c>
-      <c r="H49">
+      <c r="H49" t="n">
         <v>34.46</v>
       </c>
-      <c r="I49">
+      <c r="I49" t="n">
         <v>30.09</v>
       </c>
       <c r="J49" t="inlineStr">
@@ -1998,22 +2404,22 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D50">
+      <c r="D50" t="n">
         <v>36.37</v>
       </c>
-      <c r="E50">
+      <c r="E50" t="n">
         <v>4</v>
       </c>
-      <c r="F50">
+      <c r="F50" t="n">
         <v>26.95</v>
       </c>
-      <c r="G50">
+      <c r="G50" t="n">
         <v>4.47</v>
       </c>
-      <c r="H50">
+      <c r="H50" t="n">
         <v>35.81</v>
       </c>
-      <c r="I50">
+      <c r="I50" t="n">
         <v>25.65</v>
       </c>
       <c r="J50" t="inlineStr">
@@ -2038,22 +2444,22 @@
           <t>Automobile</t>
         </is>
       </c>
-      <c r="D51">
+      <c r="D51" t="n">
         <v>37.72</v>
       </c>
-      <c r="E51">
+      <c r="E51" t="n">
         <v>4.28</v>
       </c>
-      <c r="F51">
+      <c r="F51" t="n">
         <v>28.09</v>
       </c>
-      <c r="G51">
+      <c r="G51" t="n">
         <v>2.84</v>
       </c>
-      <c r="H51">
+      <c r="H51" t="n">
         <v>37.16</v>
       </c>
-      <c r="I51">
+      <c r="I51" t="n">
         <v>40.12</v>
       </c>
       <c r="J51" t="inlineStr">
@@ -2078,22 +2484,22 @@
           <t>Metals</t>
         </is>
       </c>
-      <c r="D52">
+      <c r="D52" t="n">
         <v>16.12</v>
       </c>
-      <c r="E52">
+      <c r="E52" t="n">
         <v>4.56</v>
       </c>
-      <c r="F52">
+      <c r="F52" t="n">
         <v>15.01</v>
       </c>
-      <c r="G52">
+      <c r="G52" t="n">
         <v>7.02</v>
       </c>
-      <c r="H52">
+      <c r="H52" t="n">
         <v>15.56</v>
       </c>
-      <c r="I52">
+      <c r="I52" t="n">
         <v>-35.25</v>
       </c>
       <c r="J52" t="inlineStr">
@@ -2118,22 +2524,22 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D53">
+      <c r="D53" t="n">
         <v>17.47</v>
       </c>
-      <c r="E53">
+      <c r="E53" t="n">
         <v>1.2</v>
       </c>
-      <c r="F53">
+      <c r="F53" t="n">
         <v>12.15</v>
       </c>
-      <c r="G53">
+      <c r="G53" t="n">
         <v>7.1</v>
       </c>
-      <c r="H53">
+      <c r="H53" t="n">
         <v>16.91</v>
       </c>
-      <c r="I53">
+      <c r="I53" t="n">
         <v>-29.83</v>
       </c>
       <c r="J53" t="inlineStr">
@@ -2158,22 +2564,22 @@
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="D54">
+      <c r="D54" t="n">
         <v>18.82</v>
       </c>
-      <c r="E54">
+      <c r="E54" t="n">
         <v>1.48</v>
       </c>
-      <c r="F54">
+      <c r="F54" t="n">
         <v>13.3</v>
       </c>
-      <c r="G54">
+      <c r="G54" t="n">
         <v>7.74</v>
       </c>
-      <c r="H54">
+      <c r="H54" t="n">
         <v>18.26</v>
       </c>
-      <c r="I54">
+      <c r="I54" t="n">
         <v>-28.29</v>
       </c>
       <c r="J54" t="inlineStr">
@@ -2198,22 +2604,22 @@
           <t>Telecom</t>
         </is>
       </c>
-      <c r="D55">
+      <c r="D55" t="n">
         <v>20.17</v>
       </c>
-      <c r="E55">
+      <c r="E55" t="n">
         <v>1.76</v>
       </c>
-      <c r="F55">
+      <c r="F55" t="n">
         <v>14.44</v>
       </c>
-      <c r="G55">
-        <v>8.88</v>
-      </c>
-      <c r="H55">
+      <c r="G55" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="H55" t="n">
         <v>19.61</v>
       </c>
-      <c r="I55">
+      <c r="I55" t="n">
         <v>-26.91</v>
       </c>
       <c r="J55" t="inlineStr">
@@ -2238,22 +2644,22 @@
           <t>Chemicals</t>
         </is>
       </c>
-      <c r="D56">
+      <c r="D56" t="n">
         <v>21.52</v>
       </c>
-      <c r="E56">
+      <c r="E56" t="n">
         <v>2.04</v>
       </c>
-      <c r="F56">
+      <c r="F56" t="n">
         <v>15.59</v>
       </c>
-      <c r="G56">
+      <c r="G56" t="n">
         <v>6.54</v>
       </c>
-      <c r="H56">
+      <c r="H56" t="n">
         <v>20.96</v>
       </c>
-      <c r="I56">
+      <c r="I56" t="n">
         <v>-25.65</v>
       </c>
       <c r="J56" t="inlineStr">
@@ -2278,22 +2684,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D57">
+      <c r="D57" t="n">
         <v>22.87</v>
       </c>
-      <c r="E57">
+      <c r="E57" t="n">
         <v>2.32</v>
       </c>
-      <c r="F57">
+      <c r="F57" t="n">
         <v>16.73</v>
       </c>
-      <c r="G57">
-        <v>5.71</v>
-      </c>
-      <c r="H57">
+      <c r="G57" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="H57" t="n">
         <v>22.31</v>
       </c>
-      <c r="I57">
+      <c r="I57" t="n">
         <v>-5.57</v>
       </c>
       <c r="J57" t="inlineStr">
@@ -2318,22 +2724,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D58">
+      <c r="D58" t="n">
         <v>24.22</v>
       </c>
-      <c r="E58">
+      <c r="E58" t="n">
         <v>2.6</v>
       </c>
-      <c r="F58">
+      <c r="F58" t="n">
         <v>17.88</v>
       </c>
-      <c r="G58">
+      <c r="G58" t="n">
         <v>6.13</v>
       </c>
-      <c r="H58">
+      <c r="H58" t="n">
         <v>23.66</v>
       </c>
-      <c r="I58">
+      <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="inlineStr">
@@ -2358,22 +2764,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D59">
+      <c r="D59" t="n">
         <v>25.57</v>
       </c>
-      <c r="E59">
+      <c r="E59" t="n">
         <v>2.88</v>
       </c>
-      <c r="F59">
+      <c r="F59" t="n">
         <v>19.02</v>
       </c>
-      <c r="G59">
+      <c r="G59" t="n">
         <v>6.17</v>
       </c>
-      <c r="H59">
+      <c r="H59" t="n">
         <v>25.01</v>
       </c>
-      <c r="I59">
+      <c r="I59" t="n">
         <v>0</v>
       </c>
       <c r="J59" t="inlineStr">
@@ -2398,22 +2804,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D60">
+      <c r="D60" t="n">
         <v>26.92</v>
       </c>
-      <c r="E60">
+      <c r="E60" t="n">
         <v>3.16</v>
       </c>
-      <c r="F60">
+      <c r="F60" t="n">
         <v>20.17</v>
       </c>
-      <c r="G60">
+      <c r="G60" t="n">
         <v>6</v>
       </c>
-      <c r="H60">
+      <c r="H60" t="n">
         <v>26.36</v>
       </c>
-      <c r="I60">
+      <c r="I60" t="n">
         <v>0</v>
       </c>
       <c r="J60" t="inlineStr">
@@ -2438,22 +2844,22 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D61">
+      <c r="D61" t="n">
         <v>28.27</v>
       </c>
-      <c r="E61">
+      <c r="E61" t="n">
         <v>3.44</v>
       </c>
-      <c r="F61">
+      <c r="F61" t="n">
         <v>21.31</v>
       </c>
-      <c r="G61">
+      <c r="G61" t="n">
         <v>3.79</v>
       </c>
-      <c r="H61">
+      <c r="H61" t="n">
         <v>27.71</v>
       </c>
-      <c r="I61">
+      <c r="I61" t="n">
         <v>-2.33</v>
       </c>
       <c r="J61" t="inlineStr">
@@ -2478,22 +2884,22 @@
           <t>Automobile</t>
         </is>
       </c>
-      <c r="D62">
+      <c r="D62" t="n">
         <v>29.62</v>
       </c>
-      <c r="E62">
+      <c r="E62" t="n">
         <v>3.72</v>
       </c>
-      <c r="F62">
+      <c r="F62" t="n">
         <v>22.46</v>
       </c>
-      <c r="G62">
+      <c r="G62" t="n">
         <v>4.12</v>
       </c>
-      <c r="H62">
+      <c r="H62" t="n">
         <v>29.06</v>
       </c>
-      <c r="I62">
+      <c r="I62" t="n">
         <v>10.03</v>
       </c>
       <c r="J62" t="inlineStr">
@@ -2518,22 +2924,22 @@
           <t>Metals</t>
         </is>
       </c>
-      <c r="D63">
+      <c r="D63" t="n">
         <v>30.97</v>
       </c>
-      <c r="E63">
+      <c r="E63" t="n">
         <v>4</v>
       </c>
-      <c r="F63">
+      <c r="F63" t="n">
         <v>23.6</v>
       </c>
-      <c r="G63">
+      <c r="G63" t="n">
         <v>4.78</v>
       </c>
-      <c r="H63">
+      <c r="H63" t="n">
         <v>30.41</v>
       </c>
-      <c r="I63">
+      <c r="I63" t="n">
         <v>24.4</v>
       </c>
       <c r="J63" t="inlineStr">
@@ -2558,22 +2964,22 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D64">
+      <c r="D64" t="n">
         <v>32.32</v>
       </c>
-      <c r="E64">
+      <c r="E64" t="n">
         <v>4.28</v>
       </c>
-      <c r="F64">
+      <c r="F64" t="n">
         <v>24.75</v>
       </c>
-      <c r="G64">
+      <c r="G64" t="n">
         <v>4.37</v>
       </c>
-      <c r="H64">
+      <c r="H64" t="n">
         <v>31.76</v>
       </c>
-      <c r="I64">
+      <c r="I64" t="n">
         <v>29.83</v>
       </c>
       <c r="J64" t="inlineStr">
@@ -2598,22 +3004,22 @@
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="D65">
+      <c r="D65" t="n">
         <v>33.67</v>
       </c>
-      <c r="E65">
+      <c r="E65" t="n">
         <v>4.56</v>
       </c>
-      <c r="F65">
+      <c r="F65" t="n">
         <v>25.89</v>
       </c>
-      <c r="G65">
+      <c r="G65" t="n">
         <v>5.14</v>
       </c>
-      <c r="H65">
+      <c r="H65" t="n">
         <v>33.11</v>
       </c>
-      <c r="I65">
+      <c r="I65" t="n">
         <v>28.29</v>
       </c>
       <c r="J65" t="inlineStr">
@@ -2638,22 +3044,22 @@
           <t>Telecom</t>
         </is>
       </c>
-      <c r="D66">
+      <c r="D66" t="n">
         <v>35.02</v>
       </c>
-      <c r="E66">
+      <c r="E66" t="n">
         <v>1.2</v>
       </c>
-      <c r="F66">
+      <c r="F66" t="n">
         <v>23.03</v>
       </c>
-      <c r="G66">
+      <c r="G66" t="n">
         <v>3.66</v>
       </c>
-      <c r="H66">
+      <c r="H66" t="n">
         <v>34.46</v>
       </c>
-      <c r="I66">
+      <c r="I66" t="n">
         <v>26.91</v>
       </c>
       <c r="J66" t="inlineStr">
@@ -2678,22 +3084,22 @@
           <t>Chemicals</t>
         </is>
       </c>
-      <c r="D67">
+      <c r="D67" t="n">
         <v>36.37</v>
       </c>
-      <c r="E67">
+      <c r="E67" t="n">
         <v>1.48</v>
       </c>
-      <c r="F67">
+      <c r="F67" t="n">
         <v>24.18</v>
       </c>
-      <c r="G67">
+      <c r="G67" t="n">
         <v>3.94</v>
       </c>
-      <c r="H67">
+      <c r="H67" t="n">
         <v>35.81</v>
       </c>
-      <c r="I67">
+      <c r="I67" t="n">
         <v>25.65</v>
       </c>
       <c r="J67" t="inlineStr">
@@ -2718,22 +3124,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D68">
+      <c r="D68" t="n">
         <v>37.72</v>
       </c>
-      <c r="E68">
+      <c r="E68" t="n">
         <v>1.76</v>
       </c>
-      <c r="F68">
+      <c r="F68" t="n">
         <v>25.32</v>
       </c>
-      <c r="G68">
+      <c r="G68" t="n">
         <v>3.99</v>
       </c>
-      <c r="H68">
+      <c r="H68" t="n">
         <v>37.16</v>
       </c>
-      <c r="I68">
+      <c r="I68" t="n">
         <v>55.74</v>
       </c>
       <c r="J68" t="inlineStr">
@@ -2758,22 +3164,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D69">
+      <c r="D69" t="n">
         <v>16.12</v>
       </c>
-      <c r="E69">
+      <c r="E69" t="n">
         <v>2.04</v>
       </c>
-      <c r="F69">
+      <c r="F69" t="n">
         <v>12.24</v>
       </c>
-      <c r="G69">
+      <c r="G69" t="n">
         <v>9.59</v>
       </c>
-      <c r="H69">
+      <c r="H69" t="n">
         <v>15.56</v>
       </c>
-      <c r="I69">
+      <c r="I69" t="n">
         <v>-33.44</v>
       </c>
       <c r="J69" t="inlineStr">
@@ -2798,22 +3204,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D70">
+      <c r="D70" t="n">
         <v>17.47</v>
       </c>
-      <c r="E70">
+      <c r="E70" t="n">
         <v>2.32</v>
       </c>
-      <c r="F70">
+      <c r="F70" t="n">
         <v>13.38</v>
       </c>
-      <c r="G70">
-        <v>9.38</v>
-      </c>
-      <c r="H70">
+      <c r="G70" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="H70" t="n">
         <v>16.91</v>
       </c>
-      <c r="I70">
+      <c r="I70" t="n">
         <v>-31.68</v>
       </c>
       <c r="J70" t="inlineStr">
@@ -2838,22 +3244,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D71">
+      <c r="D71" t="n">
         <v>18.82</v>
       </c>
-      <c r="E71">
+      <c r="E71" t="n">
         <v>2.6</v>
       </c>
-      <c r="F71">
+      <c r="F71" t="n">
         <v>14.53</v>
       </c>
-      <c r="G71">
+      <c r="G71" t="n">
         <v>4.88</v>
       </c>
-      <c r="H71">
+      <c r="H71" t="n">
         <v>18.26</v>
       </c>
-      <c r="I71">
+      <c r="I71" t="n">
         <v>-30.09</v>
       </c>
       <c r="J71" t="inlineStr">
@@ -2878,22 +3284,22 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D72">
+      <c r="D72" t="n">
         <v>20.17</v>
       </c>
-      <c r="E72">
+      <c r="E72" t="n">
         <v>2.88</v>
       </c>
-      <c r="F72">
+      <c r="F72" t="n">
         <v>15.67</v>
       </c>
-      <c r="G72">
+      <c r="G72" t="n">
         <v>5.74</v>
       </c>
-      <c r="H72">
+      <c r="H72" t="n">
         <v>19.61</v>
       </c>
-      <c r="I72">
+      <c r="I72" t="n">
         <v>-30.32</v>
       </c>
       <c r="J72" t="inlineStr">
@@ -2918,22 +3324,22 @@
           <t>Automobile</t>
         </is>
       </c>
-      <c r="D73">
+      <c r="D73" t="n">
         <v>21.52</v>
       </c>
-      <c r="E73">
+      <c r="E73" t="n">
         <v>3.16</v>
       </c>
-      <c r="F73">
+      <c r="F73" t="n">
         <v>16.82</v>
       </c>
-      <c r="G73">
+      <c r="G73" t="n">
         <v>6.78</v>
       </c>
-      <c r="H73">
+      <c r="H73" t="n">
         <v>20.96</v>
       </c>
-      <c r="I73">
+      <c r="I73" t="n">
         <v>-20.06</v>
       </c>
       <c r="J73" t="inlineStr">
@@ -2958,23 +3364,23 @@
           <t>Metals</t>
         </is>
       </c>
-      <c r="D74">
+      <c r="D74" t="n">
         <v>22.87</v>
       </c>
-      <c r="E74">
+      <c r="E74" t="n">
         <v>3.44</v>
       </c>
-      <c r="F74">
+      <c r="F74" t="n">
         <v>17.96</v>
       </c>
-      <c r="G74">
+      <c r="G74" t="n">
         <v>7.7</v>
       </c>
-      <c r="H74">
+      <c r="H74" t="n">
         <v>22.31</v>
       </c>
-      <c r="I74">
-        <v>-8.13</v>
+      <c r="I74" t="n">
+        <v>-8.130000000000001</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
@@ -2998,22 +3404,22 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D75">
+      <c r="D75" t="n">
         <v>24.22</v>
       </c>
-      <c r="E75">
+      <c r="E75" t="n">
         <v>3.72</v>
       </c>
-      <c r="F75">
+      <c r="F75" t="n">
         <v>19.11</v>
       </c>
-      <c r="G75">
-        <v>8.21</v>
-      </c>
-      <c r="H75">
+      <c r="G75" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="H75" t="n">
         <v>23.66</v>
       </c>
-      <c r="I75">
+      <c r="I75" t="n">
         <v>-2.71</v>
       </c>
       <c r="J75" t="inlineStr">
@@ -3038,22 +3444,22 @@
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="D76">
+      <c r="D76" t="n">
         <v>25.57</v>
       </c>
-      <c r="E76">
+      <c r="E76" t="n">
         <v>4</v>
       </c>
-      <c r="F76">
+      <c r="F76" t="n">
         <v>20.25</v>
       </c>
-      <c r="G76">
+      <c r="G76" t="n">
         <v>5.28</v>
       </c>
-      <c r="H76">
+      <c r="H76" t="n">
         <v>25.01</v>
       </c>
-      <c r="I76">
+      <c r="I76" t="n">
         <v>-2.57</v>
       </c>
       <c r="J76" t="inlineStr">
@@ -3078,22 +3484,22 @@
           <t>Telecom</t>
         </is>
       </c>
-      <c r="D77">
+      <c r="D77" t="n">
         <v>26.92</v>
       </c>
-      <c r="E77">
+      <c r="E77" t="n">
         <v>4.28</v>
       </c>
-      <c r="F77">
+      <c r="F77" t="n">
         <v>21.4</v>
       </c>
-      <c r="G77">
+      <c r="G77" t="n">
         <v>5.25</v>
       </c>
-      <c r="H77">
+      <c r="H77" t="n">
         <v>26.36</v>
       </c>
-      <c r="I77">
+      <c r="I77" t="n">
         <v>-2.45</v>
       </c>
       <c r="J77" t="inlineStr">
@@ -3118,22 +3524,22 @@
           <t>Chemicals</t>
         </is>
       </c>
-      <c r="D78">
+      <c r="D78" t="n">
         <v>28.27</v>
       </c>
-      <c r="E78">
+      <c r="E78" t="n">
         <v>4.56</v>
       </c>
-      <c r="F78">
+      <c r="F78" t="n">
         <v>22.54</v>
       </c>
-      <c r="G78">
+      <c r="G78" t="n">
         <v>4</v>
       </c>
-      <c r="H78">
+      <c r="H78" t="n">
         <v>27.71</v>
       </c>
-      <c r="I78">
+      <c r="I78" t="n">
         <v>-2.33</v>
       </c>
       <c r="J78" t="inlineStr">
@@ -3158,22 +3564,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D79">
+      <c r="D79" t="n">
         <v>29.62</v>
       </c>
-      <c r="E79">
+      <c r="E79" t="n">
         <v>1.2</v>
       </c>
-      <c r="F79">
+      <c r="F79" t="n">
         <v>19.68</v>
       </c>
-      <c r="G79">
+      <c r="G79" t="n">
         <v>4.22</v>
       </c>
-      <c r="H79">
+      <c r="H79" t="n">
         <v>29.06</v>
       </c>
-      <c r="I79">
+      <c r="I79" t="n">
         <v>22.3</v>
       </c>
       <c r="J79" t="inlineStr">
@@ -3198,22 +3604,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D80">
+      <c r="D80" t="n">
         <v>30.97</v>
       </c>
-      <c r="E80">
+      <c r="E80" t="n">
         <v>1.48</v>
       </c>
-      <c r="F80">
+      <c r="F80" t="n">
         <v>20.83</v>
       </c>
-      <c r="G80">
+      <c r="G80" t="n">
         <v>4.79</v>
       </c>
-      <c r="H80">
+      <c r="H80" t="n">
         <v>30.41</v>
       </c>
-      <c r="I80">
+      <c r="I80" t="n">
         <v>27.87</v>
       </c>
       <c r="J80" t="inlineStr">
@@ -3238,22 +3644,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D81">
+      <c r="D81" t="n">
         <v>32.32</v>
       </c>
-      <c r="E81">
+      <c r="E81" t="n">
         <v>1.76</v>
       </c>
-      <c r="F81">
+      <c r="F81" t="n">
         <v>21.97</v>
       </c>
-      <c r="G81">
+      <c r="G81" t="n">
         <v>3.63</v>
       </c>
-      <c r="H81">
+      <c r="H81" t="n">
         <v>31.76</v>
       </c>
-      <c r="I81">
+      <c r="I81" t="n">
         <v>26.4</v>
       </c>
       <c r="J81" t="inlineStr">
@@ -3278,22 +3684,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D82">
+      <c r="D82" t="n">
         <v>33.67</v>
       </c>
-      <c r="E82">
+      <c r="E82" t="n">
         <v>2.04</v>
       </c>
-      <c r="F82">
+      <c r="F82" t="n">
         <v>23.12</v>
       </c>
-      <c r="G82">
+      <c r="G82" t="n">
         <v>4.38</v>
       </c>
-      <c r="H82">
+      <c r="H82" t="n">
         <v>33.11</v>
       </c>
-      <c r="I82">
+      <c r="I82" t="n">
         <v>25.07</v>
       </c>
       <c r="J82" t="inlineStr">
@@ -3318,22 +3724,22 @@
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D83">
+      <c r="D83" t="n">
         <v>35.02</v>
       </c>
-      <c r="E83">
+      <c r="E83" t="n">
         <v>2.32</v>
       </c>
-      <c r="F83">
+      <c r="F83" t="n">
         <v>24.26</v>
       </c>
-      <c r="G83">
-        <v>5</v>
-      </c>
-      <c r="H83">
+      <c r="G83" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="H83" t="n">
         <v>34.46</v>
       </c>
-      <c r="I83">
+      <c r="I83" t="n">
         <v>20.99</v>
       </c>
       <c r="J83" t="inlineStr">
@@ -3358,22 +3764,22 @@
           <t>Automobile</t>
         </is>
       </c>
-      <c r="D84">
+      <c r="D84" t="n">
         <v>36.37</v>
       </c>
-      <c r="E84">
+      <c r="E84" t="n">
         <v>2.6</v>
       </c>
-      <c r="F84">
+      <c r="F84" t="n">
         <v>25.41</v>
       </c>
-      <c r="G84">
+      <c r="G84" t="n">
         <v>5.33</v>
       </c>
-      <c r="H84">
+      <c r="H84" t="n">
         <v>35.81</v>
       </c>
-      <c r="I84">
+      <c r="I84" t="n">
         <v>35.1</v>
       </c>
       <c r="J84" t="inlineStr">
@@ -3398,22 +3804,22 @@
           <t>Metals</t>
         </is>
       </c>
-      <c r="D85">
+      <c r="D85" t="n">
         <v>37.72</v>
       </c>
-      <c r="E85">
+      <c r="E85" t="n">
         <v>2.88</v>
       </c>
-      <c r="F85">
+      <c r="F85" t="n">
         <v>26.55</v>
       </c>
-      <c r="G85">
+      <c r="G85" t="n">
         <v>4.11</v>
       </c>
-      <c r="H85">
+      <c r="H85" t="n">
         <v>37.16</v>
       </c>
-      <c r="I85">
+      <c r="I85" t="n">
         <v>51.52</v>
       </c>
       <c r="J85" t="inlineStr">
@@ -3438,22 +3844,22 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D86">
+      <c r="D86" t="n">
         <v>16.12</v>
       </c>
-      <c r="E86">
+      <c r="E86" t="n">
         <v>3.16</v>
       </c>
-      <c r="F86">
+      <c r="F86" t="n">
         <v>13.47</v>
       </c>
-      <c r="G86">
+      <c r="G86" t="n">
         <v>6.29</v>
       </c>
-      <c r="H86">
+      <c r="H86" t="n">
         <v>15.56</v>
       </c>
-      <c r="I86">
+      <c r="I86" t="n">
         <v>-35.25</v>
       </c>
       <c r="J86" t="inlineStr">
@@ -3478,22 +3884,22 @@
           <t>Consumer Durables</t>
         </is>
       </c>
-      <c r="D87">
+      <c r="D87" t="n">
         <v>17.47</v>
       </c>
-      <c r="E87">
+      <c r="E87" t="n">
         <v>3.44</v>
       </c>
-      <c r="F87">
+      <c r="F87" t="n">
         <v>14.62</v>
       </c>
-      <c r="G87">
+      <c r="G87" t="n">
         <v>6.27</v>
       </c>
-      <c r="H87">
+      <c r="H87" t="n">
         <v>16.91</v>
       </c>
-      <c r="I87">
+      <c r="I87" t="n">
         <v>-33.43</v>
       </c>
       <c r="J87" t="inlineStr">
@@ -3518,22 +3924,22 @@
           <t>Telecom</t>
         </is>
       </c>
-      <c r="D88">
+      <c r="D88" t="n">
         <v>18.82</v>
       </c>
-      <c r="E88">
+      <c r="E88" t="n">
         <v>3.72</v>
       </c>
-      <c r="F88">
+      <c r="F88" t="n">
         <v>15.76</v>
       </c>
-      <c r="G88">
+      <c r="G88" t="n">
         <v>6.67</v>
       </c>
-      <c r="H88">
+      <c r="H88" t="n">
         <v>18.26</v>
       </c>
-      <c r="I88">
+      <c r="I88" t="n">
         <v>-31.8</v>
       </c>
       <c r="J88" t="inlineStr">
@@ -3558,22 +3964,22 @@
           <t>Chemicals</t>
         </is>
       </c>
-      <c r="D89">
+      <c r="D89" t="n">
         <v>20.17</v>
       </c>
-      <c r="E89">
+      <c r="E89" t="n">
         <v>4</v>
       </c>
-      <c r="F89">
+      <c r="F89" t="n">
         <v>16.91</v>
       </c>
-      <c r="G89">
+      <c r="G89" t="n">
         <v>7.58</v>
       </c>
-      <c r="H89">
+      <c r="H89" t="n">
         <v>19.61</v>
       </c>
-      <c r="I89">
+      <c r="I89" t="n">
         <v>-30.32</v>
       </c>
       <c r="J89" t="inlineStr">
@@ -3598,22 +4004,22 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D90">
+      <c r="D90" t="n">
         <v>21.52</v>
       </c>
-      <c r="E90">
+      <c r="E90" t="n">
         <v>4.28</v>
       </c>
-      <c r="F90">
+      <c r="F90" t="n">
         <v>18.05</v>
       </c>
-      <c r="G90">
-        <v>8.8</v>
-      </c>
-      <c r="H90">
+      <c r="G90" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="H90" t="n">
         <v>20.96</v>
       </c>
-      <c r="I90">
+      <c r="I90" t="n">
         <v>-11.15</v>
       </c>
       <c r="J90" t="inlineStr">
@@ -3638,22 +4044,22 @@
           <t>Financials</t>
         </is>
       </c>
-      <c r="D91">
+      <c r="D91" t="n">
         <v>22.87</v>
       </c>
-      <c r="E91">
+      <c r="E91" t="n">
         <v>4.56</v>
       </c>
-      <c r="F91">
+      <c r="F91" t="n">
         <v>19.2</v>
       </c>
-      <c r="G91">
+      <c r="G91" t="n">
         <v>6.38</v>
       </c>
-      <c r="H91">
+      <c r="H91" t="n">
         <v>22.31</v>
       </c>
-      <c r="I91">
+      <c r="I91" t="n">
         <v>-5.57</v>
       </c>
       <c r="J91" t="inlineStr">
@@ -3678,22 +4084,22 @@
           <t>FMCG</t>
         </is>
       </c>
-      <c r="D92">
+      <c r="D92" t="n">
         <v>24.22</v>
       </c>
-      <c r="E92">
+      <c r="E92" t="n">
         <v>1.2</v>
       </c>
-      <c r="F92">
+      <c r="F92" t="n">
         <v>16.34</v>
       </c>
-      <c r="G92">
+      <c r="G92" t="n">
         <v>5.41</v>
       </c>
-      <c r="H92">
+      <c r="H92" t="n">
         <v>23.66</v>
       </c>
-      <c r="I92">
+      <c r="I92" t="n">
         <v>-5.28</v>
       </c>
       <c r="J92" t="inlineStr">
@@ -3718,22 +4124,22 @@
           <t>Energy</t>
         </is>
       </c>
-      <c r="D93">
+      <c r="D93" t="n">
         <v>25.57</v>
       </c>
-      <c r="E93">
+      <c r="E93" t="n">
         <v>1.48</v>
       </c>
-      <c r="F93">
+      <c r="F93" t="n">
         <v>17.48</v>
       </c>
-      <c r="G93">
+      <c r="G93" t="n">
         <v>5.62</v>
       </c>
-      <c r="H93">
+      <c r="H93" t="n">
         <v>25.01</v>
       </c>
-      <c r="I93">
+      <c r="I93" t="n">
         <v>-5.01</v>
       </c>
       <c r="J93" t="inlineStr">
@@ -3743,5 +4149,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>